<commit_message>
Update superadmin form with category dropdown
</commit_message>
<xml_diff>
--- a/public/fcl-memories.xlsx
+++ b/public/fcl-memories.xlsx
@@ -965,8 +965,8 @@
     <col min="2" max="2" width="26.7109375" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.85546875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="106.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.28515625" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>